<commit_message>
EuroWheel ready for deploy
</commit_message>
<xml_diff>
--- a/bin/Debug/Assets/Gifts/temp_gift.xlsx
+++ b/bin/Debug/Assets/Gifts/temp_gift.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ΕΙΔΟΣ</t>
   </si>
@@ -73,12 +73,6 @@
   </si>
   <si>
     <t>ΧΟ TABLET ΠΑΙΔΙΚΟ ΜΠΛΕ</t>
-  </si>
-  <si>
-    <t>Gift 1</t>
-  </si>
-  <si>
-    <t>Gift 2</t>
   </si>
 </sst>
 </file>
@@ -520,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CB14EA-9DCF-421E-B4E0-E447C4D46EF4}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="91.83203125" customWidth="1"/>
@@ -680,16 +674,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>